<commit_message>
minor update of input data
</commit_message>
<xml_diff>
--- a/input/DatabaseCountryYear.xlsx
+++ b/input/DatabaseCountryYear.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="7">
   <si>
     <t>Country</t>
   </si>
@@ -30,6 +30,9 @@
   </si>
   <si>
     <t>2011</t>
+  </si>
+  <si>
+    <t>2021</t>
   </si>
 </sst>
 </file>
@@ -78,19 +81,19 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
-        <v>3</v>
+      <c r="B2" t="s" s="0">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixes to pass integration tests
</commit_message>
<xml_diff>
--- a/input/DatabaseCountryYear.xlsx
+++ b/input/DatabaseCountryYear.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="7">
   <si>
     <t>Country</t>
   </si>
@@ -93,7 +93,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>